<commit_message>
added sell asset button and ttested
</commit_message>
<xml_diff>
--- a/Balance Sheet/Balance Sheet - 2026.xlsx
+++ b/Balance Sheet/Balance Sheet - 2026.xlsx
@@ -435,9 +435,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:P3"/>
+  <dimension ref="B1:P7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -519,15 +520,59 @@
       <c r="P3" s="2" t="inlineStr">
         <is>
           <t>TYPE</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>07/15/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>07/15/26</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>07/15/26</t>
+        </is>
+      </c>
+      <c r="K6" t="n">
+        <v>1000</v>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>Stocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>07/15/26</t>
+        </is>
+      </c>
+      <c r="K7" t="n">
+        <v>-1000</v>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>Stocks</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="J2:L2"/>
-    <mergeCell ref="F2:H2"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="N2:P2"/>
+    <mergeCell ref="F2:H2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>